<commit_message>
Update: Rename excel upload label and add committee management features
</commit_message>
<xml_diff>
--- a/TimeTable.xlsx
+++ b/TimeTable.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity 개발\Prof-TimeTable\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Antigravity 개발\Prof-TimeTable2\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12165"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>